<commit_message>
Add supplemental repair alias groups
</commit_message>
<xml_diff>
--- a/outputs/search_phrase_taxonomy/rocket_surgery_actionable_walkthrough_taxonomy.xlsx
+++ b/outputs/search_phrase_taxonomy/rocket_surgery_actionable_walkthrough_taxonomy.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R0d67a8d8ca244c1c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Clean Actionable Phrases" sheetId="2" r:id="R77d80def9e9148b5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Taxonomy Index" sheetId="3" r:id="R1c72e4421e8e445f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Removed Non-Actionable" sheetId="4" r:id="R0dde68d21fb04887"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Methodology" sheetId="5" r:id="Ra8b4c00d1cdd439a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Rd1bd4f22854e43e6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Clean Actionable Phrases" sheetId="2" r:id="R12e00956566945b5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Taxonomy Index" sheetId="3" r:id="Rc583d2c638fe443b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Removed Non-Actionable" sheetId="4" r:id="R4b45b032c66b45bc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Methodology" sheetId="5" r:id="R54378a21dc154bfd"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -149,8 +149,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="TaxonomyIndex" displayName="TaxonomyIndex" ref="A1:K30" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A1:K30"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="TaxonomyIndex" displayName="TaxonomyIndex" ref="A1:K33" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A1:K33"/>
   <x:tableColumns count="11">
     <x:tableColumn id="1" name="Walkthrough ID"/>
     <x:tableColumn id="2" name="Canonical Query"/>
@@ -412,7 +412,7 @@
         <x:v>Generated at</x:v>
       </x:c>
       <x:c r="B4" s="6" t="str">
-        <x:v>2026-08-23 02:16:57 UTC</x:v>
+        <x:v>2026-08-23 02:29:08 UTC</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
@@ -444,7 +444,7 @@
         <x:v>Canonical walkthrough groups</x:v>
       </x:c>
       <x:c r="B8" s="6" t="n">
-        <x:v>29</x:v>
+        <x:v>32</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -6484,7 +6484,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6c4c8ce3c04249c6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc66598f2b209430f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7556,10 +7556,109 @@
         <x:v>DIY how to vacuum a heat pump system | best way to vacuum a heat pump system | can I vacuum a heat pump system myself | how to vacuum a heat pump system | how to vacuum a heat pump system for beginners | vacuum a heat pump system step by step</x:v>
       </x:c>
     </x:row>
+    <x:row r="31" ht="24" hidden="0" customHeight="1">
+      <x:c r="A31" s="9" t="str">
+        <x:v>install-dishwasher</x:v>
+      </x:c>
+      <x:c r="B31" s="9" t="str">
+        <x:v>how to install a dishwasher</x:v>
+      </x:c>
+      <x:c r="C31" s="9" t="str">
+        <x:v>Install or Replace a Dishwasher</x:v>
+      </x:c>
+      <x:c r="D31" s="9" t="str">
+        <x:v>appliances</x:v>
+      </x:c>
+      <x:c r="E31" s="9" t="str">
+        <x:v>electrical_plumbing</x:v>
+      </x:c>
+      <x:c r="F31" s="9" t="str">
+        <x:v>draft</x:v>
+      </x:c>
+      <x:c r="G31" s="9"/>
+      <x:c r="H31" s="9" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="I31" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J31" s="9" t="str">
+        <x:v>Supplemental Appliance Alias</x:v>
+      </x:c>
+      <x:c r="K31" s="9" t="str">
+        <x:v>dishwasher installation | dishwasher replacement | how to install a dishwasher | how to replace a dishwasher | install dishwasher | install a dishwasher | replace dishwasher | replace a dishwasher | replace my dishwasher</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32" ht="24" hidden="0" customHeight="1">
+      <x:c r="A32" s="9" t="str">
+        <x:v>install-window</x:v>
+      </x:c>
+      <x:c r="B32" s="9" t="str">
+        <x:v>how to install a window</x:v>
+      </x:c>
+      <x:c r="C32" s="9" t="str">
+        <x:v>Install or Replace a Window</x:v>
+      </x:c>
+      <x:c r="D32" s="9" t="str">
+        <x:v>doors_windows</x:v>
+      </x:c>
+      <x:c r="E32" s="9" t="str">
+        <x:v>standard</x:v>
+      </x:c>
+      <x:c r="F32" s="9" t="str">
+        <x:v>draft</x:v>
+      </x:c>
+      <x:c r="G32" s="9"/>
+      <x:c r="H32" s="9" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="I32" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J32" s="9" t="str">
+        <x:v>Supplemental Window Alias</x:v>
+      </x:c>
+      <x:c r="K32" s="9" t="str">
+        <x:v>add new window | correct way to put in a window | how to install a window | how to replace a window | install a new window | install a window | install new window | remove and replace old window | replace a window | replace old window</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33" ht="24" hidden="0" customHeight="1">
+      <x:c r="A33" s="9" t="str">
+        <x:v>repair-leaky-faucet</x:v>
+      </x:c>
+      <x:c r="B33" s="9" t="str">
+        <x:v>how to repair a leaky faucet</x:v>
+      </x:c>
+      <x:c r="C33" s="9" t="str">
+        <x:v>Repair a Leaky Faucet</x:v>
+      </x:c>
+      <x:c r="D33" s="9" t="str">
+        <x:v>plumbing</x:v>
+      </x:c>
+      <x:c r="E33" s="9" t="str">
+        <x:v>plumbing</x:v>
+      </x:c>
+      <x:c r="F33" s="9" t="str">
+        <x:v>draft</x:v>
+      </x:c>
+      <x:c r="G33" s="9"/>
+      <x:c r="H33" s="9" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="I33" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J33" s="9" t="str">
+        <x:v>Supplemental Plumbing Alias</x:v>
+      </x:c>
+      <x:c r="K33" s="9" t="str">
+        <x:v>fix a faucet leak | fix a leaky faucet | how to fix a leaky faucet | how to repair a leaky faucet | repair a faucet leak | repair leaky faucet | stop a faucet leak | stop a leaking faucet</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc9bd0b9cd33d4f65"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R893cc862510148bc"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -13397,7 +13496,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R75dba789287049a0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re4fd20556af14b82"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -13461,7 +13560,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfb1bbdb52e9a4895"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R935ecdbb51a540c1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add taxonomy branch selection for showers
</commit_message>
<xml_diff>
--- a/outputs/search_phrase_taxonomy/rocket_surgery_actionable_walkthrough_taxonomy.xlsx
+++ b/outputs/search_phrase_taxonomy/rocket_surgery_actionable_walkthrough_taxonomy.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Rd1bd4f22854e43e6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Clean Actionable Phrases" sheetId="2" r:id="R12e00956566945b5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Taxonomy Index" sheetId="3" r:id="Rc583d2c638fe443b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Removed Non-Actionable" sheetId="4" r:id="R4b45b032c66b45bc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Methodology" sheetId="5" r:id="R54378a21dc154bfd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Rad37ef12dc584739"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Clean Actionable Phrases" sheetId="2" r:id="R842784296c4143a7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Taxonomy Index" sheetId="3" r:id="R7ef46cdc0f6f424e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Removed Non-Actionable" sheetId="4" r:id="Rcf0b54454eac48c5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Methodology" sheetId="5" r:id="R3bc5c1f699ee4f26"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -149,8 +149,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="TaxonomyIndex" displayName="TaxonomyIndex" ref="A1:K33" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A1:K33"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="TaxonomyIndex" displayName="TaxonomyIndex" ref="A1:K34" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A1:K34"/>
   <x:tableColumns count="11">
     <x:tableColumn id="1" name="Walkthrough ID"/>
     <x:tableColumn id="2" name="Canonical Query"/>
@@ -412,7 +412,7 @@
         <x:v>Generated at</x:v>
       </x:c>
       <x:c r="B4" s="6" t="str">
-        <x:v>2026-08-23 02:29:08 UTC</x:v>
+        <x:v>2026-08-23 02:34:23 UTC</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
@@ -444,7 +444,7 @@
         <x:v>Canonical walkthrough groups</x:v>
       </x:c>
       <x:c r="B8" s="6" t="n">
-        <x:v>32</x:v>
+        <x:v>33</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -6484,7 +6484,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc66598f2b209430f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7e6300a843724ac8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7655,10 +7655,43 @@
         <x:v>fix a faucet leak | fix a leaky faucet | how to fix a leaky faucet | how to repair a leaky faucet | repair a faucet leak | repair leaky faucet | stop a faucet leak | stop a leaking faucet</x:v>
       </x:c>
     </x:row>
+    <x:row r="34" ht="24" hidden="0" customHeight="1">
+      <x:c r="A34" s="9" t="str">
+        <x:v>replace-shower</x:v>
+      </x:c>
+      <x:c r="B34" s="9" t="str">
+        <x:v>how to replace a shower</x:v>
+      </x:c>
+      <x:c r="C34" s="9" t="str">
+        <x:v>Replace a Shower</x:v>
+      </x:c>
+      <x:c r="D34" s="9" t="str">
+        <x:v>bath_shower</x:v>
+      </x:c>
+      <x:c r="E34" s="9" t="str">
+        <x:v>plumbing_waterproofing</x:v>
+      </x:c>
+      <x:c r="F34" s="9" t="str">
+        <x:v>draft</x:v>
+      </x:c>
+      <x:c r="G34" s="9"/>
+      <x:c r="H34" s="9" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="I34" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J34" s="9" t="str">
+        <x:v>Supplemental Shower Branch Alias</x:v>
+      </x:c>
+      <x:c r="K34" s="9" t="str">
+        <x:v>replace shower | replace a shower | replace my shower | remove and replace shower | install shower | install a shower | shower replacement | shower installation</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R893cc862510148bc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re267c17ff0ee4829"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -13496,7 +13529,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re4fd20556af14b82"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R284e7e5cd5e044f8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -13560,7 +13593,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R935ecdbb51a540c1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf01a6c94c9064503"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add window branch selection taxonomy
</commit_message>
<xml_diff>
--- a/outputs/search_phrase_taxonomy/rocket_surgery_actionable_walkthrough_taxonomy.xlsx
+++ b/outputs/search_phrase_taxonomy/rocket_surgery_actionable_walkthrough_taxonomy.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Rad37ef12dc584739"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Clean Actionable Phrases" sheetId="2" r:id="R842784296c4143a7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Taxonomy Index" sheetId="3" r:id="R7ef46cdc0f6f424e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Removed Non-Actionable" sheetId="4" r:id="Rcf0b54454eac48c5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Methodology" sheetId="5" r:id="R3bc5c1f699ee4f26"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R5a0fa48c95ec4883"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Clean Actionable Phrases" sheetId="2" r:id="Raf91901c91fa4a79"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Taxonomy Index" sheetId="3" r:id="R2238c32e8b864193"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Removed Non-Actionable" sheetId="4" r:id="R79feb5e742cf4fbe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Methodology" sheetId="5" r:id="R7511c2041ae648d7"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -412,7 +412,7 @@
         <x:v>Generated at</x:v>
       </x:c>
       <x:c r="B4" s="6" t="str">
-        <x:v>2026-08-23 02:34:23 UTC</x:v>
+        <x:v>2026-08-23 02:35:52 UTC</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
@@ -6484,7 +6484,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7e6300a843724ac8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R57258c3d1269458d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7691,7 +7691,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re267c17ff0ee4829"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6d1e1d5b765c49b1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -13529,7 +13529,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R284e7e5cd5e044f8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R615e120195e34d44"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -13593,7 +13593,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf01a6c94c9064503"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R71f009cb18d84d83"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>